<commit_message>
Actualizar Excel con 9 estaciones tecnicas
</commit_message>
<xml_diff>
--- a/registro_campo_carreteras.xlsx
+++ b/registro_campo_carreteras.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,14 +531,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REGISTRO TÉCNICO DE CAMPO: OBRAS DE DRENAJE, TALUDES Y GEOTECNIA VIAL</t>
+          <t>REGISTRO TÉCNICO DE CAMPO: OBRAS DE DRENAJE, TALUDES, SUELOS Y PAVIMENTOS</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Asignatura: Vías / Carreteras | Sistema de Referencia: WGS84 UTM Zona 17S | Levantamiento con Handy GPS Lite</t>
+          <t>Asignatura: Vías / Carreteras · UTPL | Sistema: WGS84 UTM Zona 17S | 9 Estaciones Georreferenciadas (Sin Duplicados)</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Sumidero de calzada con rejilla (Captación superficial)</t>
+          <t>Sumidero de calzada con rejilla (Captación superficial pluvial)</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
@@ -639,22 +639,22 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>161756.png (Rejilla), 161802.png (Talud 1), 161807.png (GPS), 161815.png (Label)</t>
+          <t>161756.png (Rejilla), 161802.png (Talud 1), 161807.png (GPS)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Coluvio / Suelo residual (Limo arenoso con grava y bloques angulosos). Grado de meteorización IV-V. Coronación con raíces expuestas y pérdida de soporte por erosión laminar.</t>
+          <t>Coluvio / Suelo residual (Limo arenoso con gravas angulosas, SUCS: SM). Grado de meteorización IV-V. Coronación con raíces expuestas por erosión laminar.</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Rejilla de hierro fundido de captación transversal en pavimento rígido de hormigón. Medida con flexómetro (~1.0 x 0.45 m). Acumulación de restos vegetales y áridos en bordillo. Se requiere limpieza preventiva.</t>
+          <t>Reja de hierro fundido de captación transversal en pavimento rígido de hormigón. Medida con flexómetro (~1.0 x 0.45 m). Acumulación de hojarasca y ramas en borde de cuneta.</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Desazolve de caja de captación, retiro de biomasa y estabilización biotecnológica de la coronación del talud.</t>
+          <t>Desazolve de caja de captación y peinado suave de coronación de talud.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Primer Punto (Talud / Calzada)</t>
+          <t>Primer Punto (Curva / Calzada)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>161823.png (Vía y talud), 161830.png (GPS), 161842.png (Anotación: 100/35 x 100)</t>
+          <t>161823.png (Vía y talud), 161830.png (GPS), 161842.png (Anotación 100/35x100)</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Corte en roca meteorizada / suelo consolidado. Pendiente de corte empinada. Relación H:V de campo registrada como 35:100 (inclinación ~70.7° o 285% de pendiente).</t>
+          <t>Corte empinado en roca meteorizada. Relación H:V = 35:100 (inclinación calculada: 70.71° / 285.71% de pendiente).</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>Calzada de pavimento rígido en curva horizontal, adecuada textura superficial estriada. Cuneta lateral al pie de talud para captación de escorrentía longitudinal.</t>
+          <t>Calzada de pavimento rígido en curva horizontal con peralte; textura estriada transversal. Cuneta lateral al pie de talud.</t>
         </is>
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>Verificar factor de seguridad del talud ante saturación y mantener despejada la cuneta al pie de corte.</t>
+          <t>Monitoreo de estabilidad ante saturación prolongada y mantenimiento de cuneta.</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Afloramiento rocoso / Talud de corte geológico</t>
+          <t>Afloramiento rocoso estratificado / foliado</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -747,22 +747,22 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>161850.png (Talud medido por brigada), 161856.png (GPS), 161902.png (Label)</t>
+          <t>161850.png (Talud medido por brigada), 161856.png (GPS)</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Macizo rocoso estratificado/foliado (posibles filitas, esquistos o areniscas limosas alteradas). Buzamiento de discontinuidades con componente hacia la vía. Alta susceptibilidad a desprendimientos.</t>
+          <t>Macizo rocoso estratificado/foliado (filitas, esquistos o areniscas limosas alteradas, Grado III-IV). Buzamiento de discontinuidades con componente hacia la vía.</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Corte verticalizado sin bermas intermedias. Presencia de vegetación pionera en el pie y bosque en la corona. Riesgo geomecánico por descompresión y meteorización diferencial.</t>
+          <t>Corte verticalizado sin banquetas intermedias. Presencia de vegetación en pie y árboles en corona. Riesgo cinemático por descompresión.</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Levantamiento estructural de diaclasas con brújula tipo Brunton (buzamiento y rumbo), perfilado de talud e instalación de malla de control de caídos si es necesario.</t>
+          <t>Levantamiento estructural de diaclasas con brújula Brunton y perfilado de talud.</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Sumidero de calzada con reja plana (Captación pluvial)</t>
+          <t>Sumidero lateral de reja plana con marco fisurado</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
@@ -801,22 +801,22 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>161909.png (Rejilla y calzada), 161915.png (GPS), 161921.png (Label)</t>
+          <t>161909.png (Rejilla y calzada), 161915.png (GPS)</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Entorno de rasante vial pavimentada. Base granular subyacente. Se observa agrietamiento en el recrecido perimetral de mortero/hormigón que confina el marco de la reja.</t>
+          <t>Rasante vial sobre base granular. Desconchamiento severo en el mortero de fijación perimetral del marco.</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>Sumidero en calzada de hormigón. Presenta fisuración del pavimento alrededor del marco por fatiga dinámica. Capacidad de captación reducida puntualmente por hojas y áridos.</t>
+          <t>Sumidero en calzada de hormigón. Presenta fisuración del pavimento alrededor del marco por impacto dinámico vehicular.</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>Reparación estructural del mortero perimetral de confinamiento mediante polímeros o microhormigón y limpieza periódica.</t>
+          <t>Reconstrucción del marco de hormigón perimetral con mortero polimérico de alta resistencia.</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Sumidero de rejilla con colmatación severa</t>
+          <t>Sumidero de rejilla severamente colmatado</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
@@ -855,22 +855,22 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>161926.png (Rejilla obstruida con basura), 161931.png (GPS), 161936.png (Label)</t>
+          <t>161926.png (Rejilla obstruida con basura), 161931.png (GPS)</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Arrastre de sedimentos aluviales/coluviales (arenas medias a gruesas, gravillas angulosas procedentes del talud lateral y berma sin confinar).</t>
+          <t>Sedimentos granulares de arrastre pluvial (arenas gruesas y gravas angulosas procedentes del talud lateral y berma).</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Obstrucción crítica (~40% del área neta) por acumulación mixta de residuos sólidos antrópicos (plásticos, cuerdas, basura) y azolve mineral. Riesgo de anegamiento en eventos de precipitación pico.</t>
+          <t>Obstrucción de aprox. 40% del área neta por basura plástica, cabos y sedimentos minerales. Reducción crítica de capacidad de captación.</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Desazolve inmediato urgente, retiro de residuos sólidos y colocación de trampa de sedimentos aguas arriba en la cuneta.</t>
+          <t>Desazolve inmediato previo a la temporada invernal y trampa de sedimentos aguas arriba.</t>
         </is>
       </c>
     </row>
@@ -880,12 +880,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Talud siguiente</t>
+          <t>Talud siguiente (Letrero Terreno)</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Talud de corte rocoso muy fracturado (Letrero 'Se Vende Terreno')</t>
+          <t>Macizo rocoso intensamente fracturado (Riesgo Rockfall)</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
@@ -909,22 +909,22 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>161943.png (Macizo rocoso fracturado), 161948.png (GPS), 161954.png (Label)</t>
+          <t>161943.png (Macizo fracturado), 161948.png (GPS)</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Macizo rocoso altamente fracturado y diaclasado (RQD bajo, Grado III-IV). Abundantes pátinas de óxido de hierro en los planos de discontinuidad. Bloques prismáticos centimétricos inestables.</t>
+          <t>Macizo rocoso altamente fracturado (RQD &lt; 25%, Grado III-IV). Pátinas de óxido de hierro en fracturas. Bloques poliédricos sueltos.</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>Frente de excavación verticalizado. Sin sistema de drenaje subsuperficial (drenes californianos) ni revestimiento. Peligro directo de caída de fragmentos rocosos sobre la vía.</t>
+          <t>Corte verticalizado sin bermas ni sostenimiento. Peligro inminente de desprendimiento de fragmentos rocosos sobre la calzada y cuneta.</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>Peinado de talud (desquinche de bloques sueltos), colocación de malla hexagonal electrosoldada o de triple torsión y zanja de coronación impermeabilizada.</t>
+          <t>Desquinche manual y colocación de malla de alambre galvanizado de triple torsión.</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Sumidero de calzada con reja (Captación lateral)</t>
+          <t>Sumidero de calzada con reja plana</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
@@ -963,7 +963,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>162005.png (GPS), 162010.png (Label), 162019.png (Rejilla e inspección brigada)</t>
+          <t>162019.png (Rejilla e inspección brigada), 162005.png (GPS)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Rejilla en servicio, ubicada en margen derecha de calzada. Colonización de vegetación en los intersticios y acumulación incipiente de sedimentos finos cohesivos.</t>
+          <t>Sumidero en servicio en margen derecha. Invasión de gramíneas en marco y depósito fino en fondo.</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Mantenimiento rutinario de limpieza y corte de vegetación perimetral para asegurar el libre ingreso de la lámina de agua.</t>
+          <t>Desbroce perimetral y limpieza periódica.</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Canal de descarga natural / Desfogue o quebrada con lodo y pencos</t>
+          <t>Canal de desfogue natural / Quebradilla colmatada por lodo</t>
         </is>
       </c>
       <c r="D12" s="7" t="n">
@@ -1017,22 +1017,76 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>162024.png (Canal/quebradilla con lodo), 162029.png (GPS), 162037.png (Label)</t>
+          <t>162024.png / WhatsApp 5.50.41 (Canal lodo), 162029.png / WhatsApp 5.50.38 (1) (GPS)</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>Suelo fino limo-arcilloso saturado (lodo plástico, alta humedad, consistencia blanda). Arrastre de sedimentos orgánicos y minerales en suspensión.</t>
+          <t>Suelo fino arcillo-limoso altamente saturado (lodo plástico, alta humedad, consistencia blanda, SUCS: CH/CL).</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>Cauce de desfogue natural de aguas pluviales colmatado severamente. Presencia de basura plástica, maleza alta y pencos (Agave). Ausencia de enrocado o encauzamiento revestido. Riesgo de taponamiento y rebose hacia la plataforma de la vía.</t>
+          <t>Cauce de desfogue natural totalmente colmatado por lodo viscoso, basura plástica y pencos (Agave americana). Alto riesgo de remanso y desborde.</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>Limpieza y rectificación del cauce de alivio, remoción de lodos y basura, conformación de cuneta de guarda o canal revestido con enrocado / gaviones en la entrega.</t>
+          <t>Dragado y perfilado de cauce, remoción de lodo y colocación de cuneta revestida o enrocado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="65" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Nueva Estación de Control (Fotos WhatsApp)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Desfogue de alcantarilla tubular con cabezal, pozos de revisión y fisuración de calzada</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>700491</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>9559201</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>2121</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>+/- 4</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>UTM WGS84 (Zona 17S)</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp 5.50.39 PM.jpeg (GPS), WhatsApp 5.50.49 PM.jpeg (Desfogue alcantarilla), WhatsApp 5.50.48 PM (2) (Pozo)</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Limo arcilloso saturado en entrega de alcantarilla y subrasante con deformaciones por humedad.</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Boca de desfogue de alcantarilla tubular de hormigón al pie de bordillo con flujo activo y vegetación hidrófila. Pozos de revisión en calzada y acera. Fisuración longitudinal de losas de hormigón y encharcamiento superficial.</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Limpieza de boca de salida de alcantarilla, sellado de fisuras en losas de pavimento y nivelación para evitar empozamientos.</t>
         </is>
       </c>
     </row>

</xml_diff>